<commit_message>
BCC platform owner on every lead notification
</commit_message>
<xml_diff>
--- a/lead-pipeline-sync.xlsx
+++ b/lead-pipeline-sync.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,39 +28,55 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000F172A"/>
+      <color rgb="001E3A8A"/>
       <sz val="18"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="0064748B"/>
+      <color rgb="006B7280"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="001E40AF"/>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005B21B6"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0092400E"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="006B21A8"/>
+      <color rgb="00065F46"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="000F172A"/>
+      <color rgb="001E3A8A"/>
       <sz val="14"/>
     </font>
     <font>
@@ -68,11 +84,22 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00991B1B"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00111827"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00065F46"/>
     </font>
   </fonts>
   <fills count="8">
@@ -84,7 +111,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F172A"/>
+        <fgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,12 +121,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00EDE9FE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E9D5FF"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,16 +150,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00D1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00D1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00D1D5DB"/>
       </bottom>
     </border>
   </borders>
@@ -146,55 +173,63 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -565,31 +600,32 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MyBidQuick — Lead Pipeline Sync</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Synced: May 11, 2026 at 06:08 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
+          <t>Synced from Supabase on May 12, 2026 at 11:10 AM UTC  •  15 leads total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>#</t>
@@ -641,273 +677,273 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Tim Sullivan</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>s.p.partyof7@gmail.com</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>9207236822</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Window Cleaning, Deck Cleaning, Gutter Cleaning</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="6" t="n">
         <v>1394</v>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Scott</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>demoarmt@gmail.com</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>4065802358</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>99 E Hyalite Peak Dr, Bozeman, MT 59718, USA</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Window Cleaning</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="6" t="n">
         <v>271</v>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Cornerstone Wash and Window Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Tim Sullivan</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>s.p.partyof7@gmail.com</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>9207236822</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Window Cleaning, Gutter Cleaning</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="6" t="n">
         <v>1533</v>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Cornerstone Wash and Window Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Jessica Wagner</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>hartmanrylee@hotmail.com</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>4065801760</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>2203 Oriole Dr, Belgrade, MT 59714, USA</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Window Cleaning</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="6" t="n">
         <v>705</v>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Cornerstone Wash and Window Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Steph Jack</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>shernandez0288@yahoo.com</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>5613088205</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>16 Fireside Dr, Bozeman, MT 59718, USA</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Window Cleaning, Gutter Cleaning</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="6" t="n">
         <v>449</v>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Cornerstone Wash and Window Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Kasey Chambers</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>kcrae2@gmail.com</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>4062076336</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>2261 Buckrake Ave, Bozeman, MT 59718, USA</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Window Cleaning, Gutter Cleaning</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="6" t="n">
         <v>231</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
@@ -915,95 +951,95 @@
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Cornerstone Wash and Window Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Steven Metellus</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>steventonice@gmail.com</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>2407841290</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>183-02 Jamaica Ave, Jamaica, NY 11423, USA</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Gutter Cleaning</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="6" t="n">
         <v>1430</v>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>County Wide Power Wash And Restorations</t>
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Tim Sullivan</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>s.p.partyof7@gmail.com</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>9207236822</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>409 Yahara St, DeForest, WI 53532, USA</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Window Cleaning</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="6" t="n">
         <v>969</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -1011,429 +1047,409 @@
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Test User</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>test@test.com</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>5551234567</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Window Cleaning</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="6" t="n">
         <v>673</v>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>test rls</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>testrls@example.com</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>6085550199</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>409 W Washington St, Chicago, IL 60606, USA</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="6" t="n">
         <v>552</v>
       </c>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>Won</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Eliott D Cloute</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>eli.cloute@clouteinc.com</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>9207231939</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>150 Majestic Vw Dr, Kalispell, MT 59901, USA</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Window Cleaning</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="6" t="n">
         <v>541</v>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Tim Sullivan</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>s.p.partyof7@gmail.com</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>9207236822</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>409 Yahara St, DeForest, WI 53532, USA</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Window Cleaning, Gutter Cleaning</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="H16" s="6" t="n">
         <v>1189</v>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Tim Sullivan</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>tim.sullivan@clouteinc.com</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>9205634101</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Pressure Washing, Window Cleaning</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="H17" s="6" t="n">
         <v>933.46</v>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Noah Baldry</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>noahbaldry34@gmail.com</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>9203972318</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>18261 MT-1, Anaconda, MT 59711, USA</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Window Cleaning</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H18" s="6" t="n">
         <v>1375</v>
       </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="32" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Test Lead - Eli Cloute</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>eli.cloute@clouteinc.com</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>9207231939</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Window Cleaning</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="H19" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>Cloute Exterior Cleaning</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Pipeline Summary</t>
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>Pipeline $</t>
-        </is>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="C25" s="14" t="n">
-        <v>7926.46</v>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Contacted</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Contacted</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="n">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C26" s="14" t="n">
-        <v>2687</v>
-      </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="B27" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" s="14" t="n">
-        <v>1200</v>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Won</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="inlineStr">
-        <is>
-          <t>Won</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Lost</t>
         </is>
       </c>
-      <c r="B29" s="13" t="n">
+      <c r="C28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>Total Pipeline (all)</t>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Total Pipeline Value</t>
         </is>
       </c>
       <c r="C30" s="20" t="n">
@@ -1441,23 +1457,23 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>Open Pipeline</t>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>Won Revenue</t>
         </is>
       </c>
       <c r="C31" s="21" t="n">
-        <v>11813.46</v>
+        <v>552</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
-        <is>
-          <t>Won Revenue</t>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>Total Leads</t>
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>552</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>